<commit_message>
Update excel-test-source-plugin plugin for v5 (#1796)
</commit_message>
<xml_diff>
--- a/excel-test-source-plugin/SampleProject/ExcelTestSource1.xlsx
+++ b/excel-test-source-plugin/SampleProject/ExcelTestSource1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\SpecSync\SpecSync\Plugins\excel-test-source-plugin\SampleProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9602969E-F46D-4F78-8B89-631AB6B80EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB6E0205-099B-44AE-8B3B-AD1D8D59C526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ExcelTestSource_ExcelTestSource" sheetId="1" r:id="rId1"/>
@@ -55,9 +55,6 @@
     <t>Test Case</t>
   </si>
   <si>
-    <t>Test Case 1 changed</t>
-  </si>
-  <si>
     <t>specsync-plugins-demo</t>
   </si>
   <si>
@@ -120,6 +117,9 @@
   </si>
   <si>
     <t>Not Automated</t>
+  </si>
+  <si>
+    <t>Test Case 1</t>
   </si>
 </sst>
 </file>
@@ -756,9 +756,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -796,7 +796,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -902,7 +902,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1044,7 +1044,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1101,16 +1101,16 @@
         <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="L1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -1121,25 +1121,25 @@
         <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="G2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" t="s">
         <v>13</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>14</v>
       </c>
-      <c r="J2" t="s">
-        <v>15</v>
-      </c>
       <c r="K2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="L2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N2">
         <v>2</v>
@@ -1150,10 +1150,10 @@
         <v>1</v>
       </c>
       <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
         <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1161,10 +1161,10 @@
         <v>2</v>
       </c>
       <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -1172,10 +1172,10 @@
         <v>3</v>
       </c>
       <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
         <v>20</v>
-      </c>
-      <c r="F5" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
@@ -1186,25 +1186,25 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" t="s">
         <v>12</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>13</v>
       </c>
-      <c r="I6" t="s">
-        <v>14</v>
-      </c>
       <c r="J6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="M6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N6">
         <v>3</v>
@@ -1215,10 +1215,10 @@
         <v>1</v>
       </c>
       <c r="E7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" t="s">
         <v>16</v>
-      </c>
-      <c r="F7" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1226,10 +1226,10 @@
         <v>2</v>
       </c>
       <c r="E8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
@@ -1237,10 +1237,10 @@
         <v>3</v>
       </c>
       <c r="E9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" t="s">
         <v>20</v>
-      </c>
-      <c r="F9" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>